<commit_message>
Upload Freezing Point Depression Module
</commit_message>
<xml_diff>
--- a/Rotation-3-Thermodynamics/Sample-Data/FreezingPointDepression_SampleData.xlsx
+++ b/Rotation-3-Thermodynamics/Sample-Data/FreezingPointDepression_SampleData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityofdallas-my.sharepoint.com/personal/pmpatel_udallas_edu/Documents/OneDrive - University of Dallas/Documents/GitHub/CHE-3131/Rotation-3-Thermodynamics/Sample-Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="72" documentId="13_ncr:1_{B2EAEA25-FDA7-40D5-A76E-DC8EAB589FD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{80055877-444F-4474-8E54-0D3A896419F1}"/>
+  <xr:revisionPtr revIDLastSave="84" documentId="13_ncr:1_{B2EAEA25-FDA7-40D5-A76E-DC8EAB589FD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C0528165-4BD7-460A-833C-D95832106A47}"/>
   <bookViews>
-    <workbookView xWindow="36120" yWindow="1980" windowWidth="23040" windowHeight="12105" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="36120" yWindow="1980" windowWidth="23040" windowHeight="12105" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pure" sheetId="3" r:id="rId1"/>
@@ -96,6 +96,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="169" formatCode="0.000"/>
+  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -143,7 +146,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -154,6 +157,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -171,6 +177,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -24707,9 +24717,10 @@
         <v>5.32</v>
       </c>
       <c r="D4" s="2">
-        <v>-1.69</v>
-      </c>
-      <c r="E4" s="2">
+        <f>C4-C2</f>
+        <v>-1.6899999999999995</v>
+      </c>
+      <c r="E4" s="6">
         <v>8.2000000000000003E-2</v>
       </c>
       <c r="F4" s="2">

</xml_diff>